<commit_message>
refactor(examples): rename assignment.xml suite to examples.xml
Rename the combined SauceDemo and DemoQA suite file to examples.xml and
its suite to ExamplesSuite, so the Extent report is written to
logs/extent-report/ExamplesSuite.html. Update the README, CHANGELOG and
master workbook references.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/main/resources/examples/testcases/Assignment_Master_Test_Cases.xlsx
+++ b/src/main/resources/examples/testcases/Assignment_Master_Test_Cases.xlsx
@@ -31,7 +31,7 @@
     <t>Run everything</t>
   </si>
   <si>
-    <t>mvn clean test "-Dsurefire.suiteXmlFiles=src/testNgXml/assignment.xml"</t>
+    <t>mvn clean test "-Dsurefire.suiteXmlFiles=src/testNgXml/examples.xml"</t>
   </si>
   <si>
     <t>Headless</t>
@@ -43,7 +43,7 @@
     <t>Extent report</t>
   </si>
   <si>
-    <t>logs/extent-report/AssignmentSuite.html</t>
+    <t>logs/extent-report/ExamplesSuite.html</t>
   </si>
   <si>
     <t>Last automated run</t>
@@ -2905,7 +2905,7 @@
     <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -6478,7 +6478,7 @@
     <mergeCell ref="A2:Q2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -6697,7 +6697,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -6891,6 +6891,6 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>